<commit_message>
finishing Grundlagen der Elektrotechnik
</commit_message>
<xml_diff>
--- a/B.Sc. LRT/Grundlagen der Elektrotechnik/images/ETech-Diagrams.xlsx
+++ b/B.Sc. LRT/Grundlagen der Elektrotechnik/images/ETech-Diagrams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Phillip\Documents\Git\Project-FoSa\B.Sc. LRT\Grundlagen der Elektrotechnik\images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77ECAB02-20F2-4CCA-BF8A-AC80DD1799AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7996C74-F03A-45B5-8574-11B2C17BB51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="18696" xr2:uid="{6006CF3B-C9F1-47C1-9F3F-D0CD89A908B6}"/>
   </bookViews>
@@ -274,10 +274,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="9.1558936816704822E-2"/>
+          <c:x val="0.14402204709758057"/>
           <c:y val="3.7592538895471282E-2"/>
-          <c:w val="0.87153472694193601"/>
-          <c:h val="0.86931343631464886"/>
+          <c:w val="0.81907162307279624"/>
+          <c:h val="0.79217811811780192"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -773,7 +773,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
@@ -912,10 +912,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.10264052544901531"/>
+          <c:x val="0.14402204709758057"/>
           <c:y val="3.7592538895471282E-2"/>
-          <c:w val="0.86045312770221116"/>
-          <c:h val="0.86931343631464886"/>
+          <c:w val="0.81907162307279624"/>
+          <c:h val="0.79217811811780192"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1116,7 +1116,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-02E6-4F6E-AC8B-8708D80D2015}"/>
+              <c16:uniqueId val="{00000001-145C-4369-B019-FDA3A5FD0EF0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1315,7 +1315,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-02E6-4F6E-AC8B-8708D80D2015}"/>
+              <c16:uniqueId val="{00000003-145C-4369-B019-FDA3A5FD0EF0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1371,7 +1371,7 @@
         <c:tickLblPos val="low"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="rnd" cmpd="sng" algn="ctr">
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="25000"/>
@@ -1387,7 +1387,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
@@ -2622,15 +2622,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>585643</xdr:colOff>
+      <xdr:colOff>771175</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>2294</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>1</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>79513</xdr:rowOff>
+      <xdr:rowOff>201</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -2645,10 +2645,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4746826" y="187824"/>
-          <a:ext cx="5775400" cy="5841915"/>
-          <a:chOff x="4723889" y="184002"/>
-          <a:chExt cx="5744819" cy="5856696"/>
+          <a:off x="4345618" y="187824"/>
+          <a:ext cx="5567009" cy="5762603"/>
+          <a:chOff x="4908438" y="184002"/>
+          <a:chExt cx="5560270" cy="5777183"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:graphicFrame macro="">
@@ -2685,8 +2685,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="6928339" y="5276658"/>
-            <a:ext cx="1831602" cy="764040"/>
+            <a:off x="6757973" y="4824943"/>
+            <a:ext cx="2476520" cy="936754"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2716,15 +2716,15 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
               </a:rPr>
-              <a:t>Zeit (Vielfache</a:t>
+              <a:t>Zeit (Vielfaches</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" baseline="0">
+              <a:rPr lang="de-DE" sz="1600" baseline="0">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -2732,7 +2732,7 @@
               <a:t> von</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -2740,14 +2740,14 @@
               <a:t> </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:latin typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
                 <a:ea typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
               </a:rPr>
               <a:t>τ</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="0">
+              <a:rPr lang="de-DE" sz="1600" i="0">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -2770,8 +2770,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm rot="16200000">
-            <a:off x="4877819" y="2557925"/>
-            <a:ext cx="1212320" cy="764038"/>
+            <a:off x="4800076" y="2355419"/>
+            <a:ext cx="1736903" cy="764038"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2801,7 +2801,7 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2812,7 +2812,7 @@
               <a:t>u</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" baseline="-25000">
+              <a:rPr lang="de-DE" sz="1600" baseline="-25000">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2823,7 +2823,7 @@
               <a:t>C</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2834,7 +2834,7 @@
               <a:t>(</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2845,7 +2845,7 @@
               <a:t>t</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2856,7 +2856,7 @@
               <a:t>)  </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -2864,7 +2864,7 @@
               <a:t>/  </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -2875,7 +2875,7 @@
               <a:t>i</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -2886,7 +2886,7 @@
               <a:t>(</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -2897,7 +2897,7 @@
               <a:t>t</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200">
+              <a:rPr lang="de-DE" sz="1600">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -2907,7 +2907,7 @@
               </a:rPr>
               <a:t>)</a:t>
             </a:r>
-            <a:endParaRPr lang="de-DE" sz="1200" i="0">
+            <a:endParaRPr lang="de-DE" sz="1600" i="0">
               <a:solidFill>
                 <a:srgbClr val="FF0000"/>
               </a:solidFill>
@@ -2931,8 +2931,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="4723889" y="250262"/>
-            <a:ext cx="877446" cy="764040"/>
+            <a:off x="4908438" y="241488"/>
+            <a:ext cx="877446" cy="779457"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -2962,7 +2962,7 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -2973,7 +2973,7 @@
               <a:t>û</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="0">
+              <a:rPr lang="de-DE" sz="1600" i="0">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -2981,7 +2981,7 @@
               <a:t> / </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -2999,16 +2999,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>702874</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>131249</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>99900</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>18606</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>789012</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>98119</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>186038</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>184258</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -3023,8 +3023,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4841120" y="5295264"/>
-          <a:ext cx="877446" cy="764040"/>
+          <a:off x="5056213" y="4776136"/>
+          <a:ext cx="881268" cy="762000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3054,7 +3054,7 @@
         <a:p>
           <a:pPr algn="ctr"/>
           <a:r>
-            <a:rPr lang="de-DE" sz="1200" i="0">
+            <a:rPr lang="de-DE" sz="1600" i="0">
               <a:solidFill>
                 <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
@@ -3072,22 +3072,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>24442</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>185529</xdr:rowOff>
+      <xdr:colOff>132522</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>2</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>83079</xdr:rowOff>
+      <xdr:colOff>1805</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>196690</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="14" name="Gruppieren 13">
+        <xdr:cNvPr id="19" name="Gruppieren 18">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74CE5006-74BC-08BB-3603-7C9A67FBEEFE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA01DE45-4564-76A6-C070-2066A30062C9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3095,442 +3095,41 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10546668" y="185529"/>
-          <a:ext cx="5727004" cy="5847776"/>
-          <a:chOff x="13939224" y="46382"/>
-          <a:chExt cx="5727004" cy="5847776"/>
+          <a:off x="10045148" y="185530"/>
+          <a:ext cx="5620727" cy="5762603"/>
+          <a:chOff x="10654748" y="185530"/>
+          <a:chExt cx="5620727" cy="5762603"/>
         </a:xfrm>
       </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="13" name="Gruppieren 12">
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="16" name="Diagramm 15">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E66CE3F7-F8E7-F1E6-AF8D-34BC95F3D52F}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FAAC6C4-83CC-4422-8382-C1286DC491F3}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="13939224" y="46382"/>
-            <a:ext cx="5727004" cy="5847776"/>
-            <a:chOff x="11101753" y="181708"/>
-            <a:chExt cx="5855537" cy="5862557"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:grpSp>
-          <xdr:nvGrpSpPr>
-            <xdr:cNvPr id="5" name="Gruppieren 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54BD9650-46CE-42D7-9806-71B88E250C5A}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGrpSpPr/>
-          </xdr:nvGrpSpPr>
-          <xdr:grpSpPr>
-            <a:xfrm>
-              <a:off x="11101753" y="181708"/>
-              <a:ext cx="5855537" cy="5862557"/>
-              <a:chOff x="4564449" y="-613167"/>
-              <a:chExt cx="5659315" cy="5862557"/>
-            </a:xfrm>
-          </xdr:grpSpPr>
-          <xdr:graphicFrame macro="">
-            <xdr:nvGraphicFramePr>
-              <xdr:cNvPr id="6" name="Diagramm 5">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D66BA3EC-E905-87FA-C05C-DF2BA298A56E}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvGraphicFramePr/>
-            </xdr:nvGraphicFramePr>
-            <xdr:xfrm>
-              <a:off x="4725320" y="-613167"/>
-              <a:ext cx="5498444" cy="5777182"/>
-            </xdr:xfrm>
-            <a:graphic>
-              <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-                <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-              </a:graphicData>
-            </a:graphic>
-          </xdr:graphicFrame>
-          <xdr:sp macro="" textlink="">
-            <xdr:nvSpPr>
-              <xdr:cNvPr id="7" name="Textfeld 6">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B50260A3-A6C7-9BDF-AAE7-027329C51669}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvSpPr txBox="1"/>
-            </xdr:nvSpPr>
-            <xdr:spPr>
-              <a:xfrm>
-                <a:off x="6795619" y="4485350"/>
-                <a:ext cx="1734412" cy="764040"/>
-              </a:xfrm>
-              <a:prstGeom prst="rect">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:noFill/>
-              <a:ln w="9525" cmpd="sng">
-                <a:noFill/>
-              </a:ln>
-            </xdr:spPr>
-            <xdr:style>
-              <a:lnRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:lnRef>
-              <a:fillRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:fillRef>
-              <a:effectRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:effectRef>
-              <a:fontRef idx="minor">
-                <a:schemeClr val="dk1"/>
-              </a:fontRef>
-            </xdr:style>
-            <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr algn="ctr"/>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>Zeit (Vielfache von </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:latin typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
-                    <a:ea typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
-                  </a:rPr>
-                  <a:t>τ</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="0">
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>)</a:t>
-                </a:r>
-              </a:p>
-            </xdr:txBody>
-          </xdr:sp>
-          <xdr:sp macro="" textlink="">
-            <xdr:nvSpPr>
-              <xdr:cNvPr id="8" name="Textfeld 7">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8EEDBE6-274E-C569-2536-56163CF37A81}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvSpPr txBox="1"/>
-            </xdr:nvSpPr>
-            <xdr:spPr>
-              <a:xfrm rot="16200000">
-                <a:off x="4661338" y="1004618"/>
-                <a:ext cx="1212320" cy="764038"/>
-              </a:xfrm>
-              <a:prstGeom prst="rect">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:noFill/>
-              <a:ln w="9525" cmpd="sng">
-                <a:noFill/>
-              </a:ln>
-            </xdr:spPr>
-            <xdr:style>
-              <a:lnRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:lnRef>
-              <a:fillRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:fillRef>
-              <a:effectRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:effectRef>
-              <a:fontRef idx="minor">
-                <a:schemeClr val="dk1"/>
-              </a:fontRef>
-            </xdr:style>
-            <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr algn="ctr"/>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>u</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" baseline="-25000">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>C</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>(</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>t</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>)  </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>/  </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>i</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>(</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>t</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>)</a:t>
-                </a:r>
-                <a:endParaRPr lang="de-DE" sz="1200" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="FF0000"/>
-                  </a:solidFill>
-                  <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                </a:endParaRPr>
-              </a:p>
-            </xdr:txBody>
-          </xdr:sp>
-          <xdr:sp macro="" textlink="">
-            <xdr:nvSpPr>
-              <xdr:cNvPr id="9" name="Textfeld 8">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB6BA167-4BAE-7F4E-8342-C760943E5F67}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvSpPr txBox="1"/>
-            </xdr:nvSpPr>
-            <xdr:spPr>
-              <a:xfrm>
-                <a:off x="4564449" y="-541046"/>
-                <a:ext cx="877446" cy="764040"/>
-              </a:xfrm>
-              <a:prstGeom prst="rect">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:noFill/>
-              <a:ln w="9525" cmpd="sng">
-                <a:noFill/>
-              </a:ln>
-            </xdr:spPr>
-            <xdr:style>
-              <a:lnRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:lnRef>
-              <a:fillRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:fillRef>
-              <a:effectRef idx="0">
-                <a:scrgbClr r="0" g="0" b="0"/>
-              </a:effectRef>
-              <a:fontRef idx="minor">
-                <a:schemeClr val="dk1"/>
-              </a:fontRef>
-            </xdr:style>
-            <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr algn="ctr"/>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="086FBD"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>û</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="0">
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t> / </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="de-DE" sz="1200" i="1">
-                    <a:solidFill>
-                      <a:srgbClr val="FF0000"/>
-                    </a:solidFill>
-                    <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                    <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  </a:rPr>
-                  <a:t>î</a:t>
-                </a:r>
-              </a:p>
-            </xdr:txBody>
-          </xdr:sp>
-        </xdr:grpSp>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="12" name="Textfeld 11">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1AA0435-1707-43E7-A062-36EB60FA263C}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11247782" y="2780664"/>
-              <a:ext cx="877446" cy="764040"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln w="9525" cmpd="sng">
-              <a:noFill/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="dk1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr algn="ctr"/>
-              <a:r>
-                <a:rPr lang="de-DE" sz="1200" i="0">
-                  <a:solidFill>
-                    <a:sysClr val="windowText" lastClr="000000"/>
-                  </a:solidFill>
-                  <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                  <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
-                </a:rPr>
-                <a:t>0</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </xdr:grpSp>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="10707757" y="185530"/>
+          <a:ext cx="5567718" cy="5762603"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="10" name="Textfeld 9">
+          <xdr:cNvPr id="7" name="Textfeld 6">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0A63665-0F62-4F1B-B1C0-1155C54A5483}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B50260A3-A6C7-9BDF-AAE7-027329C51669}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -3538,8 +3137,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="14020495" y="5107440"/>
-            <a:ext cx="713630" cy="762000"/>
+            <a:off x="12576315" y="4813990"/>
+            <a:ext cx="2473698" cy="997087"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -3569,7 +3168,370 @@
           <a:p>
             <a:pPr algn="ctr"/>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600">
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>Zeit (Vielfaches von </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:latin typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
+                <a:ea typeface="Latin Modern Math" panose="02000503000000000000" pitchFamily="50" charset="0"/>
+              </a:rPr>
+              <a:t>τ</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="0">
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="Textfeld 7">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8EEDBE6-274E-C569-2536-56163CF37A81}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="16200000">
+            <a:off x="10561404" y="1509457"/>
+            <a:ext cx="1724749" cy="773176"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>u</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" baseline="-25000">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>C</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>t</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>)  </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600">
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>/  </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>i</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>(</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>t</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>)</a:t>
+            </a:r>
+            <a:endParaRPr lang="de-DE" sz="1600" i="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="9" name="Textfeld 8">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB6BA167-4BAE-7F4E-8342-C760943E5F67}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10725573" y="225287"/>
+            <a:ext cx="887941" cy="774417"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="086FBD"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>û</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="0">
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t> / </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>î</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="Textfeld 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1AA0435-1707-43E7-A062-36EB60FA263C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10861770" y="2511286"/>
+            <a:ext cx="858185" cy="737211"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+                <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
+              </a:rPr>
+              <a:t>0</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="10" name="Textfeld 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0A63665-0F62-4F1B-B1C0-1155C54A5483}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10654748" y="4797287"/>
+            <a:ext cx="852473" cy="747474"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="086FBD"/>
                 </a:solidFill>
@@ -3580,7 +3542,7 @@
               <a:t>-û</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="0">
+              <a:rPr lang="de-DE" sz="1600" i="0">
                 <a:latin typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:ea typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
                 <a:cs typeface="CMU Serif" panose="02000603000000000000" pitchFamily="2" charset="0"/>
@@ -3588,7 +3550,7 @@
               <a:t> / </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="0">
+              <a:rPr lang="de-DE" sz="1600" i="0">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -3599,7 +3561,7 @@
               <a:t>-</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="de-DE" sz="1200" i="1">
+              <a:rPr lang="de-DE" sz="1600" i="1">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -3939,6 +3901,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="7" max="7" width="2.6640625" customWidth="1"/>
     <col min="15" max="15" width="2.6640625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>